<commit_message>
Elite Upgrade: Synchronized Dashboard, Ultimate Analysis Guide, and inclusive stock screening
</commit_message>
<xml_diff>
--- a/portfolio_aom_analysis_report.xlsx
+++ b/portfolio_aom_analysis_report.xlsx
@@ -873,16 +873,16 @@
         <v>14.66666666666669</v>
       </c>
       <c r="Q4" t="n">
-        <v>65.53333333333333</v>
+        <v>71.53333333333333</v>
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>Wait/Hold</t>
+          <t>Buy More</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>Keep Holding</t>
+          <t>Wait &amp; Bid @ 18.27</t>
         </is>
       </c>
       <c r="T4" t="n">
@@ -1079,7 +1079,7 @@
         <v>6.611570247933876</v>
       </c>
       <c r="Q6" t="n">
-        <v>60.33884297520661</v>
+        <v>54.33884297520661</v>
       </c>
       <c r="R6" t="inlineStr">
         <is>
@@ -1285,7 +1285,7 @@
         <v>29.62962962962964</v>
       </c>
       <c r="Q8" t="n">
-        <v>46.03703703703704</v>
+        <v>52.03703703703704</v>
       </c>
       <c r="R8" t="inlineStr">
         <is>
@@ -1491,7 +1491,7 @@
         <v>45.45454545454543</v>
       </c>
       <c r="Q10" t="n">
-        <v>44.45454545454545</v>
+        <v>38.45454545454545</v>
       </c>
       <c r="R10" t="inlineStr">
         <is>
@@ -1697,7 +1697,7 @@
         <v>67.49999999999999</v>
       </c>
       <c r="Q12" t="n">
-        <v>66.75</v>
+        <v>60.75</v>
       </c>
       <c r="R12" t="inlineStr">
         <is>
@@ -2315,7 +2315,7 @@
         <v>29.09090909090912</v>
       </c>
       <c r="Q18" t="n">
-        <v>83.59090909090909</v>
+        <v>77.59090909090909</v>
       </c>
       <c r="R18" t="inlineStr">
         <is>

</xml_diff>